<commit_message>
chore: update SD-WAN CVE report [2026-06-30]
</commit_message>
<xml_diff>
--- a/docs/sdwan_report.xlsx
+++ b/docs/sdwan_report.xlsx
@@ -14,7 +14,7 @@
     <sheet name="Fortinet" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Citrix" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Versa Networks" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="VMware" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Arista" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Palo Alto Networks" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Juniper" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Cradlepoint" sheetId="11" state="visible" r:id="rId11"/>
@@ -1868,7 +1868,7 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
@@ -5798,7 +5798,7 @@
       </c>
       <c r="F69" s="19" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G69" s="20" t="inlineStr">
@@ -6990,7 +6990,7 @@
       </c>
       <c r="F103" s="19" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G103" s="20" t="inlineStr">
@@ -8707,7 +8707,7 @@
       </c>
       <c r="F152" s="19" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G152" s="20" t="inlineStr">
@@ -9535,7 +9535,7 @@
       </c>
       <c r="F176" s="19" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G176" s="20" t="inlineStr">
@@ -11171,7 +11171,7 @@
       </c>
       <c r="F224" s="19" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G224" s="20" t="inlineStr">
@@ -13230,7 +13230,7 @@
       </c>
       <c r="F282" s="25" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G282" s="26" t="inlineStr">
@@ -17367,7 +17367,7 @@
       </c>
       <c r="F400" s="25" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G400" s="26" t="inlineStr">
@@ -18145,7 +18145,7 @@
       </c>
       <c r="F422" s="25" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G422" s="26" t="inlineStr">
@@ -35811,7 +35811,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="39" t="inlineStr">
         <is>
-          <t>VMware  |  SD-WAN CVE Analysis</t>
+          <t>Arista  |  SD-WAN CVE Analysis</t>
         </is>
       </c>
     </row>
@@ -36076,7 +36076,7 @@
     <row r="71" ht="20" customHeight="1">
       <c r="A71" s="8" t="inlineStr">
         <is>
-          <t>VMware — Individual CVEs (8 total, sorted by severity)</t>
+          <t>Arista — Individual CVEs (8 total, sorted by severity)</t>
         </is>
       </c>
     </row>
@@ -36143,7 +36143,7 @@
       </c>
       <c r="F73" s="19" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G73" s="20" t="inlineStr">
@@ -36178,7 +36178,7 @@
       </c>
       <c r="F74" s="19" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G74" s="20" t="inlineStr">
@@ -36213,7 +36213,7 @@
       </c>
       <c r="F75" s="19" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G75" s="20" t="inlineStr">
@@ -36248,7 +36248,7 @@
       </c>
       <c r="F76" s="19" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G76" s="20" t="inlineStr">
@@ -36286,7 +36286,7 @@
       </c>
       <c r="F77" s="19" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G77" s="20" t="inlineStr">
@@ -36325,7 +36325,7 @@
       </c>
       <c r="F78" s="25" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G78" s="26" t="inlineStr">
@@ -36360,7 +36360,7 @@
       </c>
       <c r="F79" s="25" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G79" s="26" t="inlineStr">
@@ -36398,7 +36398,7 @@
       </c>
       <c r="F80" s="25" t="inlineStr">
         <is>
-          <t>VMware</t>
+          <t>Arista</t>
         </is>
       </c>
       <c r="G80" s="26" t="inlineStr">

</xml_diff>